<commit_message>
Upgrade master study hub to 24 Encyclopedic Handwritten Modules covering full Advanced Excel curriculum, shortcuts, error debugging, and 100 case studies
</commit_message>
<xml_diff>
--- a/Excel Formulas .xlsx
+++ b/Excel Formulas .xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucky\Desktop\Advance Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00F5FB19-61BE-4111-91E0-3E33A674F916}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E895E4B2-4C86-4428-9238-37FFA47D68E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12720" tabRatio="913" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" tabRatio="913" firstSheet="14" activeTab="14" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IF FORMULA" sheetId="15" r:id="rId1"/>
@@ -46,6 +46,17 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -59,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="693" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="803" uniqueCount="333">
   <si>
     <t>Ashok Singh</t>
   </si>
@@ -403,9 +414,6 @@
     <t>SALARY</t>
   </si>
   <si>
-    <t>&gt;=20000</t>
-  </si>
-  <si>
     <t>LEFT</t>
   </si>
   <si>
@@ -649,9 +657,6 @@
     <t>first last</t>
   </si>
   <si>
-    <t>First</t>
-  </si>
-  <si>
     <t>last</t>
   </si>
   <si>
@@ -794,13 +799,283 @@
   </si>
   <si>
     <t>or</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>barack</t>
+  </si>
+  <si>
+    <t>george</t>
+  </si>
+  <si>
+    <t>william</t>
+  </si>
+  <si>
+    <t>ronald</t>
+  </si>
+  <si>
+    <t>james</t>
+  </si>
+  <si>
+    <t>gerald</t>
+  </si>
+  <si>
+    <t>richard</t>
+  </si>
+  <si>
+    <t>lyndon</t>
+  </si>
+  <si>
+    <t>john</t>
+  </si>
+  <si>
+    <t>dwight</t>
+  </si>
+  <si>
+    <t>harry</t>
+  </si>
+  <si>
+    <t>franklin</t>
+  </si>
+  <si>
+    <t>herbert</t>
+  </si>
+  <si>
+    <t>calvin</t>
+  </si>
+  <si>
+    <t>warren</t>
+  </si>
+  <si>
+    <t>woodrow</t>
+  </si>
+  <si>
+    <t>theodore</t>
+  </si>
+  <si>
+    <t>benjamin</t>
+  </si>
+  <si>
+    <t>grover</t>
+  </si>
+  <si>
+    <t>chester</t>
+  </si>
+  <si>
+    <t>rutherford</t>
+  </si>
+  <si>
+    <t>ulysses</t>
+  </si>
+  <si>
+    <t>andrew</t>
+  </si>
+  <si>
+    <t>abraham</t>
+  </si>
+  <si>
+    <t>hussein</t>
+  </si>
+  <si>
+    <t>walker</t>
+  </si>
+  <si>
+    <t>jefferson</t>
+  </si>
+  <si>
+    <t>wilson</t>
+  </si>
+  <si>
+    <t>earl</t>
+  </si>
+  <si>
+    <t>rudolph</t>
+  </si>
+  <si>
+    <t>milhous</t>
+  </si>
+  <si>
+    <t>baines</t>
+  </si>
+  <si>
+    <t>fitzgerald</t>
+  </si>
+  <si>
+    <t>david</t>
+  </si>
+  <si>
+    <t>s</t>
+  </si>
+  <si>
+    <t>delano</t>
+  </si>
+  <si>
+    <t>clark</t>
+  </si>
+  <si>
+    <t>coolidge</t>
+  </si>
+  <si>
+    <t>gamaliel</t>
+  </si>
+  <si>
+    <t>howard</t>
+  </si>
+  <si>
+    <t>roosevelt</t>
+  </si>
+  <si>
+    <t>mckinley</t>
+  </si>
+  <si>
+    <t>harrison</t>
+  </si>
+  <si>
+    <t>cleveland</t>
+  </si>
+  <si>
+    <t>alan</t>
+  </si>
+  <si>
+    <t>abram</t>
+  </si>
+  <si>
+    <t>birchard</t>
+  </si>
+  <si>
+    <t>simpson</t>
+  </si>
+  <si>
+    <t>johnson</t>
+  </si>
+  <si>
+    <t>lincoln</t>
+  </si>
+  <si>
+    <t>Column1</t>
+  </si>
+  <si>
+    <t>Column2</t>
+  </si>
+  <si>
+    <t>Column3</t>
+  </si>
+  <si>
+    <t>first</t>
+  </si>
+  <si>
+    <t>millard</t>
+  </si>
+  <si>
+    <t>zachary</t>
+  </si>
+  <si>
+    <t>martin</t>
+  </si>
+  <si>
+    <t>thomas</t>
+  </si>
+  <si>
+    <t>buchanan</t>
+  </si>
+  <si>
+    <t>pierce</t>
+  </si>
+  <si>
+    <t>fillmore</t>
+  </si>
+  <si>
+    <t>taylor</t>
+  </si>
+  <si>
+    <t>knox</t>
+  </si>
+  <si>
+    <t>tyler</t>
+  </si>
+  <si>
+    <t>henry</t>
+  </si>
+  <si>
+    <t>van</t>
+  </si>
+  <si>
+    <t>jackson</t>
+  </si>
+  <si>
+    <t>quincy</t>
+  </si>
+  <si>
+    <t>monroe</t>
+  </si>
+  <si>
+    <t>madison</t>
+  </si>
+  <si>
+    <t>adams</t>
+  </si>
+  <si>
+    <t>washington</t>
+  </si>
+  <si>
+    <t>ABC</t>
+  </si>
+  <si>
+    <t>HTG</t>
+  </si>
+  <si>
+    <t>RSF</t>
+  </si>
+  <si>
+    <t>IUW</t>
+  </si>
+  <si>
+    <t>GFD</t>
+  </si>
+  <si>
+    <t>HPK</t>
+  </si>
+  <si>
+    <t>TDG</t>
+  </si>
+  <si>
+    <t>OHI</t>
+  </si>
+  <si>
+    <t>MOI</t>
+  </si>
+  <si>
+    <t>HGF</t>
+  </si>
+  <si>
+    <t>IKJ</t>
+  </si>
+  <si>
+    <t>AVS</t>
+  </si>
+  <si>
+    <t>ERR</t>
+  </si>
+  <si>
+    <t>UJH</t>
+  </si>
+  <si>
+    <t>OKJ</t>
+  </si>
+  <si>
+    <t>PLK</t>
+  </si>
+  <si>
+    <t>SDG</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="16">
+  <numFmts count="17">
     <numFmt numFmtId="8" formatCode="&quot;₹&quot;\ #,##0.00;[Red]&quot;₹&quot;\ \-#,##0.00"/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="164" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
@@ -817,6 +1092,7 @@
     <numFmt numFmtId="175" formatCode="dd"/>
     <numFmt numFmtId="176" formatCode="dddd"/>
     <numFmt numFmtId="177" formatCode="[Green][&gt;=25000]General;[Red][&lt;25000]General"/>
+    <numFmt numFmtId="178" formatCode="[$-F800]dddd\,\ mmmm\ dd\,\ yyyy"/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -1104,7 +1380,7 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -1137,7 +1413,6 @@
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1167,8 +1442,25 @@
     <xf numFmtId="43" fontId="4" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
-    <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="8" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1184,21 +1476,6 @@
     <xf numFmtId="0" fontId="9" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -1208,6 +1485,26 @@
     <cellStyle name="Percent" xfId="4" builtinId="5"/>
   </cellStyles>
   <dxfs count="8">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -1325,26 +1622,6 @@
         <top/>
         <bottom/>
       </border>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1512,8 +1789,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="1813891" y="688939"/>
-          <a:ext cx="5419442" cy="1811711"/>
+          <a:off x="1797326" y="720588"/>
+          <a:ext cx="5259457" cy="1871869"/>
           <a:chOff x="1794184" y="723444"/>
           <a:chExt cx="5151498" cy="1911283"/>
         </a:xfrm>
@@ -1693,12 +1970,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="sk" displayName="sk" ref="A1:C16" totalsRowShown="0" headerRowDxfId="5" headerRowBorderDxfId="4" tableBorderDxfId="3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="sk" displayName="sk" ref="A1:C16" totalsRowShown="0" headerRowDxfId="7" headerRowBorderDxfId="6" tableBorderDxfId="5">
   <autoFilter ref="A1:C16" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Employee Code" dataDxfId="2"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Designation" dataDxfId="1"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Salary" dataDxfId="0" dataCellStyle="Percent"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Employee Code" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Designation" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Salary" dataDxfId="2" dataCellStyle="Percent"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{9CF168E9-4D08-4E74-967F-C543096C5C45}" name="Table2" displayName="Table2" ref="A1:C45" totalsRowShown="0">
+  <autoFilter ref="A1:C45" xr:uid="{9CF168E9-4D08-4E74-967F-C543096C5C45}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{5080066C-35DA-4242-8CB5-AC60CAC2A935}" name="Column1"/>
+    <tableColumn id="2" xr3:uid="{5E8B9742-071D-48D7-8513-9D83F9EAFB1D}" name="Column2"/>
+    <tableColumn id="3" xr3:uid="{94E86564-6129-49A8-A0F8-B523BE6BBBBB}" name="Column3"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1989,11 +2278,17 @@
       <c r="D1" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="E1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H1" s="22" t="s">
         <v>112</v>
       </c>
-      <c r="I1" s="23" t="s">
-        <v>211</v>
+      <c r="I1" s="22" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
@@ -2006,12 +2301,23 @@
       <c r="C2" s="1">
         <v>15000</v>
       </c>
-      <c r="D2" s="51"/>
+      <c r="D2" s="49" t="str">
+        <f>IF(C2&gt;$H$2,$I$2,"No")</f>
+        <v>No</v>
+      </c>
+      <c r="E2" s="49">
+        <f>IF(C2&gt;$H$2,$I$5,$I$6)</f>
+        <v>0.05</v>
+      </c>
+      <c r="F2" s="50">
+        <f>IF(C2&gt;$H$2,$I$8,$I$9)</f>
+        <v>500</v>
+      </c>
       <c r="H2">
         <v>20000</v>
       </c>
       <c r="I2" t="s">
-        <v>198</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -2024,9 +2330,20 @@
       <c r="C3" s="1">
         <v>16000</v>
       </c>
-      <c r="D3" s="51"/>
+      <c r="D3" s="49" t="str">
+        <f t="shared" ref="D3:D13" si="0">IF(C3&gt;$H$2,$I$2,"No")</f>
+        <v>No</v>
+      </c>
+      <c r="E3" s="49">
+        <f t="shared" ref="E3:E13" si="1">IF(C3&gt;$H$2,$I$5,$I$6)</f>
+        <v>0.05</v>
+      </c>
+      <c r="F3" s="50">
+        <f t="shared" ref="F3:F13" si="2">IF(C3&gt;$H$2,$I$8,$I$9)</f>
+        <v>500</v>
+      </c>
       <c r="I3" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -2039,7 +2356,18 @@
       <c r="C4" s="1">
         <v>18000</v>
       </c>
-      <c r="D4" s="51"/>
+      <c r="D4" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v>No</v>
+      </c>
+      <c r="E4" s="49">
+        <f t="shared" si="1"/>
+        <v>0.05</v>
+      </c>
+      <c r="F4" s="50">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -2051,11 +2379,22 @@
       <c r="C5" s="1">
         <v>19000</v>
       </c>
-      <c r="D5" s="51"/>
+      <c r="D5" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v>No</v>
+      </c>
+      <c r="E5" s="49">
+        <f t="shared" si="1"/>
+        <v>0.05</v>
+      </c>
+      <c r="F5" s="50">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
       <c r="H5" t="s">
-        <v>240</v>
-      </c>
-      <c r="I5" s="25">
+        <v>238</v>
+      </c>
+      <c r="I5" s="24">
         <v>0.1</v>
       </c>
     </row>
@@ -2069,8 +2408,19 @@
       <c r="C6" s="1">
         <v>25000</v>
       </c>
-      <c r="D6" s="51"/>
-      <c r="I6" s="25">
+      <c r="D6" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v>Yes</v>
+      </c>
+      <c r="E6" s="49">
+        <f t="shared" si="1"/>
+        <v>0.1</v>
+      </c>
+      <c r="F6" s="50">
+        <f t="shared" si="2"/>
+        <v>1000</v>
+      </c>
+      <c r="I6" s="24">
         <v>0.05</v>
       </c>
     </row>
@@ -2084,7 +2434,18 @@
       <c r="C7" s="1">
         <v>22000</v>
       </c>
-      <c r="D7" s="51"/>
+      <c r="D7" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v>Yes</v>
+      </c>
+      <c r="E7" s="49">
+        <f t="shared" si="1"/>
+        <v>0.1</v>
+      </c>
+      <c r="F7" s="50">
+        <f t="shared" si="2"/>
+        <v>1000</v>
+      </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
@@ -2096,9 +2457,20 @@
       <c r="C8" s="1">
         <v>15000</v>
       </c>
-      <c r="D8" s="51"/>
+      <c r="D8" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v>No</v>
+      </c>
+      <c r="E8" s="49">
+        <f t="shared" si="1"/>
+        <v>0.05</v>
+      </c>
+      <c r="F8" s="50">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
       <c r="H8" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="I8">
         <v>1000</v>
@@ -2114,7 +2486,18 @@
       <c r="C9" s="1">
         <v>35000</v>
       </c>
-      <c r="D9" s="51"/>
+      <c r="D9" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v>Yes</v>
+      </c>
+      <c r="E9" s="49">
+        <f t="shared" si="1"/>
+        <v>0.1</v>
+      </c>
+      <c r="F9" s="50">
+        <f t="shared" si="2"/>
+        <v>1000</v>
+      </c>
       <c r="I9">
         <v>500</v>
       </c>
@@ -2129,7 +2512,18 @@
       <c r="C10" s="1">
         <v>15000</v>
       </c>
-      <c r="D10" s="51"/>
+      <c r="D10" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v>No</v>
+      </c>
+      <c r="E10" s="49">
+        <f t="shared" si="1"/>
+        <v>0.05</v>
+      </c>
+      <c r="F10" s="50">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
@@ -2141,7 +2535,18 @@
       <c r="C11" s="1">
         <v>35000</v>
       </c>
-      <c r="D11" s="51"/>
+      <c r="D11" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v>Yes</v>
+      </c>
+      <c r="E11" s="49">
+        <f t="shared" si="1"/>
+        <v>0.1</v>
+      </c>
+      <c r="F11" s="50">
+        <f t="shared" si="2"/>
+        <v>1000</v>
+      </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
@@ -2153,7 +2558,18 @@
       <c r="C12" s="1">
         <v>18000</v>
       </c>
-      <c r="D12" s="51"/>
+      <c r="D12" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v>No</v>
+      </c>
+      <c r="E12" s="49">
+        <f t="shared" si="1"/>
+        <v>0.05</v>
+      </c>
+      <c r="F12" s="50">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
@@ -2165,7 +2581,18 @@
       <c r="C13" s="1">
         <v>21000</v>
       </c>
-      <c r="D13" s="51"/>
+      <c r="D13" s="49" t="str">
+        <f t="shared" si="0"/>
+        <v>Yes</v>
+      </c>
+      <c r="E13" s="49">
+        <f t="shared" si="1"/>
+        <v>0.1</v>
+      </c>
+      <c r="F13" s="50">
+        <f t="shared" si="2"/>
+        <v>1000</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2199,7 +2626,7 @@
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="41">
+      <c r="A2" s="40">
         <v>43740</v>
       </c>
       <c r="B2" t="s">
@@ -2213,7 +2640,7 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="41">
+      <c r="A3" s="40">
         <v>43742</v>
       </c>
       <c r="B3" t="s">
@@ -2227,7 +2654,7 @@
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="41">
+      <c r="A4" s="40">
         <v>43745</v>
       </c>
       <c r="B4" t="s">
@@ -2241,7 +2668,7 @@
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="41">
+      <c r="A5" s="40">
         <v>43746</v>
       </c>
       <c r="B5" t="s">
@@ -2255,7 +2682,7 @@
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="41">
+      <c r="A6" s="40">
         <v>43744</v>
       </c>
       <c r="B6" t="s">
@@ -2269,7 +2696,7 @@
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="41">
+      <c r="A7" s="40">
         <v>43747</v>
       </c>
       <c r="B7" t="s">
@@ -2283,7 +2710,7 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="41">
+      <c r="A8" s="40">
         <v>44062</v>
       </c>
       <c r="B8" t="s">
@@ -2297,7 +2724,7 @@
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="41">
+      <c r="A9" s="40">
         <v>43750</v>
       </c>
       <c r="B9" t="s">
@@ -2311,7 +2738,7 @@
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="41">
+      <c r="A10" s="40">
         <v>43739</v>
       </c>
       <c r="B10" t="s">
@@ -2325,7 +2752,7 @@
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="41">
+      <c r="A11" s="40">
         <v>43741</v>
       </c>
       <c r="B11" t="s">
@@ -2339,7 +2766,7 @@
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="41">
+      <c r="A12" s="40">
         <v>43743</v>
       </c>
       <c r="B12" t="s">
@@ -2353,7 +2780,7 @@
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="41">
+      <c r="A13" s="40">
         <v>43749</v>
       </c>
       <c r="B13" t="s">
@@ -2395,8 +2822,8 @@
       <c r="D1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="E1" t="s">
-        <v>204</v>
+      <c r="E1" s="3" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -2412,8 +2839,12 @@
       <c r="D2" s="1">
         <v>450</v>
       </c>
+      <c r="E2">
+        <f>SUMPRODUCT(C2,D2)</f>
+        <v>225000</v>
+      </c>
       <c r="G2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -2429,6 +2860,10 @@
       <c r="D3" s="1">
         <v>950</v>
       </c>
+      <c r="E3">
+        <f t="shared" ref="E3:E13" si="0">SUMPRODUCT(C3,D3)</f>
+        <v>570000</v>
+      </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -2443,6 +2878,10 @@
       <c r="D4" s="1">
         <v>350</v>
       </c>
+      <c r="E4">
+        <f t="shared" si="0"/>
+        <v>157500</v>
+      </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -2457,11 +2896,15 @@
       <c r="D5" s="1">
         <v>350</v>
       </c>
+      <c r="E5">
+        <f t="shared" si="0"/>
+        <v>122500</v>
+      </c>
       <c r="G5" s="3" t="s">
         <v>110</v>
       </c>
       <c r="H5" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -2477,11 +2920,15 @@
       <c r="D6" s="1">
         <v>250</v>
       </c>
+      <c r="E6">
+        <f t="shared" si="0"/>
+        <v>162500</v>
+      </c>
       <c r="G6" s="1" t="s">
         <v>54</v>
       </c>
       <c r="I6" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -2497,8 +2944,12 @@
       <c r="D7" s="1">
         <v>850</v>
       </c>
+      <c r="E7">
+        <f t="shared" si="0"/>
+        <v>102000</v>
+      </c>
       <c r="I7" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -2514,6 +2965,10 @@
       <c r="D8" s="1">
         <v>3500</v>
       </c>
+      <c r="E8">
+        <f t="shared" si="0"/>
+        <v>875000</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -2528,6 +2983,10 @@
       <c r="D9" s="1">
         <v>2500</v>
       </c>
+      <c r="E9">
+        <f t="shared" si="0"/>
+        <v>375000</v>
+      </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -2542,6 +3001,10 @@
       <c r="D10" s="1">
         <v>2500</v>
       </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>625000</v>
+      </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
@@ -2556,6 +3019,10 @@
       <c r="D11" s="1">
         <v>3500</v>
       </c>
+      <c r="E11">
+        <f t="shared" si="0"/>
+        <v>1260000</v>
+      </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
@@ -2570,6 +3037,10 @@
       <c r="D12" s="1">
         <v>1800</v>
       </c>
+      <c r="E12">
+        <f t="shared" si="0"/>
+        <v>216000</v>
+      </c>
       <c r="G12" s="3" t="s">
         <v>110</v>
       </c>
@@ -2577,7 +3048,7 @@
         <v>111</v>
       </c>
       <c r="I12" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -2593,19 +3064,23 @@
       <c r="D13" s="1">
         <v>1200</v>
       </c>
+      <c r="E13">
+        <f t="shared" si="0"/>
+        <v>252000</v>
+      </c>
       <c r="G13" s="1" t="s">
         <v>54</v>
       </c>
       <c r="H13" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="K13" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="K14" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2622,9 +3097,9 @@
     <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="19.7109375" customWidth="1"/>
     <col min="4" max="4" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="6.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.85546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.85546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="18.28515625" bestFit="1" customWidth="1"/>
   </cols>
@@ -2634,264 +3109,408 @@
         <v>65</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>115</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>116</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>66</v>
       </c>
+      <c r="E2" t="str">
+        <f>LEFT(D2,6)</f>
+        <v>Mumbai</v>
+      </c>
+      <c r="F2" t="str">
+        <f>RIGHT(D2,3)</f>
+        <v>086</v>
+      </c>
+      <c r="G2" t="str">
+        <f>MID(D2,4,7)</f>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>67</v>
       </c>
+      <c r="E3" t="str">
+        <f t="shared" ref="E3:E13" si="0">LEFT(D3,6)</f>
+        <v>Mumbai</v>
+      </c>
+      <c r="F3" t="str">
+        <f t="shared" ref="F3:F13" si="1">RIGHT(D3,3)</f>
+        <v>087</v>
+      </c>
+      <c r="G3" t="str">
+        <f t="shared" ref="G3:G13" si="2">MID(D3,4,7)</f>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>68</v>
       </c>
+      <c r="E4" t="str">
+        <f t="shared" si="0"/>
+        <v>Mumbai</v>
+      </c>
+      <c r="F4" t="str">
+        <f t="shared" si="1"/>
+        <v>088</v>
+      </c>
+      <c r="G4" t="str">
+        <f t="shared" si="2"/>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>69</v>
       </c>
+      <c r="E5" t="str">
+        <f t="shared" si="0"/>
+        <v>Mumbai</v>
+      </c>
+      <c r="F5" t="str">
+        <f t="shared" si="1"/>
+        <v>089</v>
+      </c>
+      <c r="G5" t="str">
+        <f t="shared" si="2"/>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>70</v>
       </c>
+      <c r="E6" t="str">
+        <f t="shared" si="0"/>
+        <v>Mumbai</v>
+      </c>
+      <c r="F6" t="str">
+        <f t="shared" si="1"/>
+        <v>090</v>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" si="2"/>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>71</v>
       </c>
+      <c r="E7" t="str">
+        <f t="shared" si="0"/>
+        <v>Mumbai</v>
+      </c>
+      <c r="F7" t="str">
+        <f t="shared" si="1"/>
+        <v>091</v>
+      </c>
+      <c r="G7" t="str">
+        <f t="shared" si="2"/>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>72</v>
       </c>
+      <c r="E8" t="str">
+        <f t="shared" si="0"/>
+        <v>Mumbai</v>
+      </c>
+      <c r="F8" t="str">
+        <f t="shared" si="1"/>
+        <v>092</v>
+      </c>
+      <c r="G8" t="str">
+        <f t="shared" si="2"/>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>73</v>
       </c>
+      <c r="E9" t="str">
+        <f t="shared" si="0"/>
+        <v>Mumbai</v>
+      </c>
+      <c r="F9" t="str">
+        <f t="shared" si="1"/>
+        <v>093</v>
+      </c>
+      <c r="G9" t="str">
+        <f t="shared" si="2"/>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>74</v>
       </c>
+      <c r="E10" t="str">
+        <f t="shared" si="0"/>
+        <v>Mumbai</v>
+      </c>
+      <c r="F10" t="str">
+        <f t="shared" si="1"/>
+        <v>094</v>
+      </c>
+      <c r="G10" t="str">
+        <f t="shared" si="2"/>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>75</v>
       </c>
+      <c r="E11" t="str">
+        <f t="shared" si="0"/>
+        <v>Mumbai</v>
+      </c>
+      <c r="F11" t="str">
+        <f t="shared" si="1"/>
+        <v>095</v>
+      </c>
+      <c r="G11" t="str">
+        <f t="shared" si="2"/>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>76</v>
       </c>
+      <c r="E12" t="str">
+        <f t="shared" si="0"/>
+        <v>Mumbai</v>
+      </c>
+      <c r="F12" t="str">
+        <f t="shared" si="1"/>
+        <v>096</v>
+      </c>
+      <c r="G12" t="str">
+        <f t="shared" si="2"/>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>77</v>
       </c>
+      <c r="E13" t="str">
+        <f t="shared" si="0"/>
+        <v>Mumbai</v>
+      </c>
+      <c r="F13" t="str">
+        <f t="shared" si="1"/>
+        <v>097</v>
+      </c>
+      <c r="G13" t="str">
+        <f t="shared" si="2"/>
+        <v>bai -40</v>
+      </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>
@@ -2902,7 +3521,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-1000-000000000000}">
-  <dimension ref="A1:G44"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
@@ -2911,293 +3530,667 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>195</v>
+        <v>294</v>
       </c>
       <c r="B1" t="s">
-        <v>196</v>
+        <v>295</v>
       </c>
       <c r="C1" t="s">
-        <v>197</v>
+        <v>296</v>
       </c>
       <c r="E1" s="12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F1" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="G1" s="12" t="s">
         <v>135</v>
-      </c>
-      <c r="G1" s="12" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>152</v>
+        <v>194</v>
+      </c>
+      <c r="B2" t="s">
+        <v>297</v>
+      </c>
+      <c r="C2" t="s">
+        <v>195</v>
       </c>
       <c r="E2" t="s">
-        <v>118</v>
+        <v>117</v>
+      </c>
+      <c r="F2" t="s">
+        <v>316</v>
+      </c>
+      <c r="G2">
+        <v>986</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>153</v>
+        <v>151</v>
+      </c>
+      <c r="B3" t="s">
+        <v>244</v>
+      </c>
+      <c r="C3" t="s">
+        <v>268</v>
       </c>
       <c r="E3" t="s">
-        <v>119</v>
+        <v>118</v>
+      </c>
+      <c r="F3" t="s">
+        <v>317</v>
+      </c>
+      <c r="G3">
+        <v>987</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>154</v>
+        <v>152</v>
+      </c>
+      <c r="B4" t="s">
+        <v>245</v>
+      </c>
+      <c r="C4" t="s">
+        <v>269</v>
       </c>
       <c r="E4" t="s">
-        <v>120</v>
+        <v>119</v>
+      </c>
+      <c r="F4">
+        <v>985</v>
+      </c>
+      <c r="G4" t="s">
+        <v>325</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>155</v>
+        <v>153</v>
+      </c>
+      <c r="B5" t="s">
+        <v>246</v>
+      </c>
+      <c r="C5" t="s">
+        <v>270</v>
       </c>
       <c r="E5" t="s">
-        <v>121</v>
+        <v>120</v>
+      </c>
+      <c r="F5">
+        <v>748</v>
+      </c>
+      <c r="G5" t="s">
+        <v>326</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>156</v>
+        <v>154</v>
+      </c>
+      <c r="B6" t="s">
+        <v>245</v>
+      </c>
+      <c r="C6" t="s">
+        <v>256</v>
       </c>
       <c r="E6" t="s">
-        <v>122</v>
+        <v>121</v>
+      </c>
+      <c r="F6" t="s">
+        <v>318</v>
+      </c>
+      <c r="G6">
+        <v>854</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>157</v>
+        <v>155</v>
+      </c>
+      <c r="B7" t="s">
+        <v>247</v>
+      </c>
+      <c r="C7" t="s">
+        <v>271</v>
       </c>
       <c r="E7" t="s">
-        <v>123</v>
+        <v>122</v>
+      </c>
+      <c r="F7" t="s">
+        <v>319</v>
+      </c>
+      <c r="G7">
+        <v>965</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>158</v>
+        <v>156</v>
+      </c>
+      <c r="B8" t="s">
+        <v>248</v>
+      </c>
+      <c r="C8" t="s">
+        <v>272</v>
       </c>
       <c r="E8" t="s">
-        <v>124</v>
+        <v>123</v>
+      </c>
+      <c r="F8">
+        <v>655</v>
+      </c>
+      <c r="G8" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>159</v>
+        <v>157</v>
+      </c>
+      <c r="B9" t="s">
+        <v>249</v>
+      </c>
+      <c r="C9" t="s">
+        <v>273</v>
       </c>
       <c r="E9" t="s">
-        <v>125</v>
+        <v>124</v>
+      </c>
+      <c r="F9">
+        <v>321</v>
+      </c>
+      <c r="G9" t="s">
+        <v>328</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>160</v>
+        <v>158</v>
+      </c>
+      <c r="B10" t="s">
+        <v>250</v>
+      </c>
+      <c r="C10" t="s">
+        <v>274</v>
       </c>
       <c r="E10" t="s">
-        <v>126</v>
+        <v>125</v>
+      </c>
+      <c r="F10" t="s">
+        <v>320</v>
+      </c>
+      <c r="G10">
+        <v>955</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>161</v>
+        <v>159</v>
+      </c>
+      <c r="B11" t="s">
+        <v>251</v>
+      </c>
+      <c r="C11" t="s">
+        <v>275</v>
       </c>
       <c r="E11" t="s">
-        <v>127</v>
+        <v>126</v>
+      </c>
+      <c r="F11">
+        <v>965</v>
+      </c>
+      <c r="G11" t="s">
+        <v>329</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>162</v>
+        <v>160</v>
+      </c>
+      <c r="B12" t="s">
+        <v>252</v>
+      </c>
+      <c r="C12" t="s">
+        <v>276</v>
       </c>
       <c r="E12" t="s">
-        <v>128</v>
+        <v>127</v>
+      </c>
+      <c r="F12" t="s">
+        <v>321</v>
+      </c>
+      <c r="G12">
+        <v>965</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>163</v>
+        <v>161</v>
+      </c>
+      <c r="B13" t="s">
+        <v>253</v>
+      </c>
+      <c r="C13" t="s">
+        <v>277</v>
       </c>
       <c r="E13" t="s">
-        <v>129</v>
+        <v>128</v>
+      </c>
+      <c r="F13">
+        <v>857</v>
+      </c>
+      <c r="G13" t="s">
+        <v>330</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>164</v>
+        <v>162</v>
+      </c>
+      <c r="B14" t="s">
+        <v>254</v>
+      </c>
+      <c r="C14" t="s">
+        <v>278</v>
       </c>
       <c r="E14" t="s">
-        <v>130</v>
+        <v>129</v>
+      </c>
+      <c r="F14">
+        <v>965</v>
+      </c>
+      <c r="G14" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>165</v>
+        <v>163</v>
+      </c>
+      <c r="B15" t="s">
+        <v>255</v>
+      </c>
+      <c r="C15" t="s">
+        <v>279</v>
       </c>
       <c r="E15" t="s">
-        <v>131</v>
+        <v>130</v>
+      </c>
+      <c r="F15">
+        <v>147</v>
+      </c>
+      <c r="G15" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>164</v>
+      </c>
+      <c r="B16" t="s">
+        <v>256</v>
+      </c>
+      <c r="C16" t="s">
+        <v>280</v>
+      </c>
+      <c r="E16" t="s">
+        <v>131</v>
+      </c>
+      <c r="F16" t="s">
+        <v>322</v>
+      </c>
+      <c r="G16">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>165</v>
+      </c>
+      <c r="B17" t="s">
+        <v>257</v>
+      </c>
+      <c r="C17" t="s">
+        <v>281</v>
+      </c>
+      <c r="E17" t="s">
+        <v>132</v>
+      </c>
+      <c r="F17" t="s">
+        <v>323</v>
+      </c>
+      <c r="G17">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
         <v>166</v>
       </c>
-      <c r="E16" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="B18" t="s">
+        <v>258</v>
+      </c>
+      <c r="C18" t="s">
+        <v>282</v>
+      </c>
+      <c r="E18" t="s">
+        <v>133</v>
+      </c>
+      <c r="F18" t="s">
+        <v>324</v>
+      </c>
+      <c r="G18">
+        <v>974</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
         <v>167</v>
       </c>
-      <c r="E17" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="B19" t="s">
+        <v>259</v>
+      </c>
+      <c r="C19" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
         <v>168</v>
       </c>
-      <c r="E18" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="B20" t="s">
+        <v>246</v>
+      </c>
+      <c r="C20" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="B21" t="s">
+        <v>260</v>
+      </c>
+      <c r="C21" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="B22" t="s">
+        <v>246</v>
+      </c>
+      <c r="C22" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="B23" t="s">
+        <v>261</v>
+      </c>
+      <c r="C23" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="B24" t="s">
+        <v>262</v>
+      </c>
+      <c r="C24" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="B25" t="s">
+        <v>263</v>
+      </c>
+      <c r="C25" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+      <c r="B26" t="s">
+        <v>248</v>
+      </c>
+      <c r="C26" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+      <c r="B27" t="s">
+        <v>264</v>
+      </c>
+      <c r="C27" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+      <c r="B28" t="s">
+        <v>265</v>
+      </c>
+      <c r="C28" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+      <c r="B29" t="s">
+        <v>266</v>
+      </c>
+      <c r="C29" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
         <v>178</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+      <c r="B30" t="s">
+        <v>267</v>
+      </c>
+      <c r="C30" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+      <c r="B31" t="s">
+        <v>248</v>
+      </c>
+      <c r="C31" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+      <c r="B32" t="s">
+        <v>255</v>
+      </c>
+      <c r="C32" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+      <c r="B33" t="s">
+        <v>298</v>
+      </c>
+      <c r="C33" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+      <c r="B34" t="s">
+        <v>299</v>
+      </c>
+      <c r="C34" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="B35" t="s">
+        <v>248</v>
+      </c>
+      <c r="C35" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
         <v>184</v>
       </c>
-    </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+      <c r="B36" t="s">
+        <v>252</v>
+      </c>
+      <c r="C36" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+      <c r="B37" t="s">
+        <v>246</v>
+      </c>
+      <c r="C37" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+      <c r="B38" t="s">
+        <v>300</v>
+      </c>
+      <c r="C38" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>187</v>
       </c>
-    </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+      <c r="B39" t="s">
+        <v>266</v>
+      </c>
+      <c r="C39" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+      <c r="B40" t="s">
+        <v>252</v>
+      </c>
+      <c r="C40" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
         <v>189</v>
       </c>
-    </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+      <c r="B41" t="s">
+        <v>248</v>
+      </c>
+      <c r="C41" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
         <v>190</v>
       </c>
-    </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+      <c r="B42" t="s">
+        <v>248</v>
+      </c>
+      <c r="C42" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
         <v>191</v>
       </c>
-    </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+      <c r="B43" t="s">
+        <v>301</v>
+      </c>
+      <c r="C43" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
         <v>192</v>
       </c>
-    </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+      <c r="B44" t="s">
+        <v>252</v>
+      </c>
+      <c r="C44" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
         <v>193</v>
       </c>
-    </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>194</v>
+      <c r="B45" t="s">
+        <v>245</v>
+      </c>
+      <c r="C45" t="s">
+        <v>315</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -3211,10 +4204,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
+      <c r="A1" s="61" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="56"/>
+      <c r="B1" s="62"/>
       <c r="C1" s="18"/>
       <c r="D1" s="18"/>
       <c r="E1" s="18"/>
@@ -3231,25 +4224,37 @@
       <c r="A3" s="20" t="s">
         <v>104</v>
       </c>
-      <c r="B3" s="20"/>
+      <c r="B3" s="20" t="str">
+        <f>SUBSTITUTE(A3,"-","")</f>
+        <v>9812345678</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="20" t="s">
         <v>103</v>
       </c>
-      <c r="B4" s="20"/>
+      <c r="B4" s="20" t="str">
+        <f>SUBSTITUTE(A4,",","-")</f>
+        <v>MUMBAI- 400086</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="20" t="s">
         <v>102</v>
       </c>
-      <c r="B5" s="20"/>
+      <c r="B5" s="20" t="str">
+        <f>SUBSTITUTE(A5,"-","_")</f>
+        <v>9812_12_12_12</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="20" t="s">
         <v>101</v>
       </c>
-      <c r="B6" s="20"/>
+      <c r="B6" s="20" t="str">
+        <f>SUBSTITUTE(A6,","," ")</f>
+        <v>DELHI 400001</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3283,10 +4288,10 @@
       <c r="A1" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="57" t="s">
+      <c r="B1" s="53" t="s">
         <v>100</v>
       </c>
-      <c r="C1" s="58"/>
+      <c r="C1" s="54"/>
       <c r="F1" s="13" t="s">
         <v>87</v>
       </c>
@@ -3299,14 +4304,14 @@
       <c r="I1" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="K1" s="59" t="s">
+      <c r="K1" s="55" t="s">
         <v>97</v>
       </c>
-      <c r="L1" s="60"/>
-      <c r="N1" s="61" t="s">
+      <c r="L1" s="56"/>
+      <c r="N1" s="57" t="s">
         <v>96</v>
       </c>
-      <c r="O1" s="61"/>
+      <c r="O1" s="57"/>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
@@ -3318,13 +4323,25 @@
       <c r="F2" s="1">
         <v>1</v>
       </c>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
+      <c r="G2" s="7">
+        <f>IPMT($C$3/12,F2,$C$5,-$C$4)</f>
+        <v>833.33333333333337</v>
+      </c>
+      <c r="H2" s="7">
+        <f>PPMT($C$3,F2,$C$5,-$C$4)</f>
+        <v>6274.5394882511609</v>
+      </c>
+      <c r="I2" s="7">
+        <f>PMT($C$3,$C$5,-$C$4)</f>
+        <v>16274.539488251161</v>
+      </c>
       <c r="K2" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="L2" s="1"/>
+      <c r="L2" s="52">
+        <f>PV(L3,L5,-L4)</f>
+        <v>199343.14594370543</v>
+      </c>
       <c r="N2" s="1"/>
       <c r="O2" s="1"/>
     </row>
@@ -3347,9 +4364,18 @@
       <c r="F3" s="1">
         <v>2</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
+      <c r="G3" s="7">
+        <f t="shared" ref="G3:G11" si="0">IPMT($C$3/12,F3,$C$5,-$C$4)</f>
+        <v>753.07746028662052</v>
+      </c>
+      <c r="H3" s="7">
+        <f t="shared" ref="H3:H11" si="1">PPMT($C$3,F3,$C$5,-$C$4)</f>
+        <v>6901.9934370762776</v>
+      </c>
+      <c r="I3" s="7">
+        <f t="shared" ref="I3:I11" si="2">PMT($C$3,$C$5,-$C$4)</f>
+        <v>16274.539488251161</v>
+      </c>
       <c r="K3" s="1" t="s">
         <v>91</v>
       </c>
@@ -3379,9 +4405,18 @@
       <c r="F4" s="1">
         <v>3</v>
       </c>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
+      <c r="G4" s="7">
+        <f t="shared" si="0"/>
+        <v>672.15278829785188</v>
+      </c>
+      <c r="H4" s="7">
+        <f t="shared" si="1"/>
+        <v>7592.1927807839056</v>
+      </c>
+      <c r="I4" s="7">
+        <f t="shared" si="2"/>
+        <v>16274.539488251161</v>
+      </c>
       <c r="K4" s="1" t="s">
         <v>83</v>
       </c>
@@ -3411,9 +4446,18 @@
       <c r="F5" s="1">
         <v>4</v>
       </c>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
-      <c r="I5" s="7"/>
+      <c r="G5" s="7">
+        <f t="shared" si="0"/>
+        <v>590.55374404251017</v>
+      </c>
+      <c r="H5" s="7">
+        <f t="shared" si="1"/>
+        <v>8351.4120588622955</v>
+      </c>
+      <c r="I5" s="7">
+        <f t="shared" si="2"/>
+        <v>16274.539488251161</v>
+      </c>
       <c r="K5" s="1" t="s">
         <v>85</v>
       </c>
@@ -3432,9 +4476,18 @@
       <c r="F6" s="1">
         <v>5</v>
       </c>
-      <c r="G6" s="7"/>
-      <c r="H6" s="7"/>
-      <c r="I6" s="7"/>
+      <c r="G6" s="7">
+        <f t="shared" si="0"/>
+        <v>508.2747077517073</v>
+      </c>
+      <c r="H6" s="7">
+        <f t="shared" si="1"/>
+        <v>9186.5532647485252</v>
+      </c>
+      <c r="I6" s="7">
+        <f t="shared" si="2"/>
+        <v>16274.539488251161</v>
+      </c>
     </row>
     <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
@@ -3447,17 +4500,32 @@
       <c r="F7" s="1">
         <v>6</v>
       </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="7"/>
-      <c r="I7" s="7"/>
+      <c r="G7" s="7">
+        <f t="shared" si="0"/>
+        <v>425.31001282514779</v>
+      </c>
+      <c r="H7" s="7">
+        <f t="shared" si="1"/>
+        <v>10105.208591223378</v>
+      </c>
+      <c r="I7" s="7">
+        <f t="shared" si="2"/>
+        <v>16274.539488251161</v>
+      </c>
       <c r="K7" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="L7" s="9"/>
+      <c r="L7" s="52">
+        <f>PV(L3,L5,-L4)</f>
+        <v>199343.14594370543</v>
+      </c>
       <c r="N7" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="O7" s="9"/>
+      <c r="O7" s="9">
+        <f>FV(O3,O5,-O4)</f>
+        <v>78056.16258846609</v>
+      </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
@@ -3471,9 +4539,18 @@
       <c r="F8" s="1">
         <v>7</v>
       </c>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
-      <c r="I8" s="7"/>
+      <c r="G8" s="7">
+        <f t="shared" si="0"/>
+        <v>341.65394544086683</v>
+      </c>
+      <c r="H8" s="7">
+        <f t="shared" si="1"/>
+        <v>11115.729450345716</v>
+      </c>
+      <c r="I8" s="7">
+        <f t="shared" si="2"/>
+        <v>16274.539488251161</v>
+      </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
@@ -3487,47 +4564,86 @@
       <c r="F9" s="1">
         <v>8</v>
       </c>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
-      <c r="I9" s="7"/>
+      <c r="G9" s="7">
+        <f t="shared" si="0"/>
+        <v>257.30074416171698</v>
+      </c>
+      <c r="H9" s="7">
+        <f t="shared" si="1"/>
+        <v>12227.302395380288</v>
+      </c>
+      <c r="I9" s="7">
+        <f t="shared" si="2"/>
+        <v>16274.539488251161</v>
+      </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F10" s="1">
         <v>9</v>
       </c>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
-      <c r="I10" s="7"/>
+      <c r="G10" s="7">
+        <f t="shared" si="0"/>
+        <v>172.24459953857416</v>
+      </c>
+      <c r="H10" s="7">
+        <f t="shared" si="1"/>
+        <v>13450.032634918316</v>
+      </c>
+      <c r="I10" s="7">
+        <f t="shared" si="2"/>
+        <v>16274.539488251161</v>
+      </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C11" s="6"/>
       <c r="F11" s="1">
         <v>10</v>
       </c>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
-      <c r="I11" s="7"/>
+      <c r="G11" s="7">
+        <f t="shared" si="0"/>
+        <v>86.47965371023848</v>
+      </c>
+      <c r="H11" s="7">
+        <f t="shared" si="1"/>
+        <v>14795.035898410146</v>
+      </c>
+      <c r="I11" s="7">
+        <f t="shared" si="2"/>
+        <v>16274.539488251161</v>
+      </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="F12" s="1"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
+      <c r="G12" s="7">
+        <f>SUM(G2:G11)</f>
+        <v>4640.3809893885682</v>
+      </c>
+      <c r="H12" s="7">
+        <f>SUM(H2:H11)</f>
+        <v>100000</v>
+      </c>
+      <c r="I12" s="7">
+        <f>SUM(I2:I11)</f>
+        <v>162745.39488251158</v>
+      </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="H14" s="17"/>
+      <c r="H14" s="17">
+        <f>I12-H12</f>
+        <v>62745.39488251158</v>
+      </c>
     </row>
     <row r="18" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D18" s="42"/>
+      <c r="D18" s="41"/>
     </row>
     <row r="20" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D20" s="43"/>
+      <c r="D20" s="42"/>
     </row>
     <row r="24" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D24" s="25"/>
+      <c r="D24" s="24"/>
     </row>
     <row r="25" spans="4:4" x14ac:dyDescent="0.25">
-      <c r="D25" s="43"/>
+      <c r="D25" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3546,52 +4662,51 @@
   <dimension ref="A1:F40"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="3" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="3" width="15.42578125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="41">
+      <c r="A3" s="40">
         <f ca="1">TODAY()</f>
-        <v>46252</v>
+        <v>46277</v>
       </c>
       <c r="B3">
         <v>7</v>
       </c>
-      <c r="C3" s="41">
+      <c r="C3" s="40">
         <f ca="1">A3+B3</f>
-        <v>46259</v>
+        <v>46284</v>
       </c>
       <c r="D3" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" s="41">
+      <c r="A4" s="40">
         <f ca="1">TODAY()</f>
-        <v>46252</v>
+        <v>46277</v>
       </c>
       <c r="B4">
         <v>5</v>
       </c>
-      <c r="C4" s="41">
+      <c r="C4" s="40">
         <f ca="1">A4-B4</f>
-        <v>46247</v>
+        <v>46272</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="50">
+      <c r="A6" s="40">
         <f ca="1">NOW()</f>
-        <v>46252.847921875</v>
+        <v>46277.878781712963</v>
       </c>
       <c r="C6" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -3600,95 +4715,95 @@
         <v>2026</v>
       </c>
       <c r="C8" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9">
         <f ca="1">MONTH(A6)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C9" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <f ca="1">DAY(A6)</f>
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="C10" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A12" s="41">
+      <c r="A12" s="40">
         <f ca="1">DATE(A8,A9,A10)</f>
-        <v>46252</v>
+        <v>46277</v>
       </c>
       <c r="C12" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="41"/>
+      <c r="A13" s="40"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="str">
         <f ca="1">TEXT(A6,"dddd")</f>
-        <v>Tuesday</v>
+        <v>Saturday</v>
       </c>
       <c r="B14" t="str">
         <f ca="1">TEXT(A6,"mmmm")</f>
-        <v>August</v>
+        <v>September</v>
       </c>
       <c r="C14" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="str">
         <f ca="1">TEXT(A12,"ddd")</f>
-        <v>Tue</v>
+        <v>Sat</v>
       </c>
       <c r="B15" t="str">
         <f ca="1">TEXT(A6,"mmm")</f>
-        <v>Aug</v>
+        <v>Sep</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f ca="1">TEXT(A12,"dd")</f>
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="B16" t="str">
         <f ca="1">TEXT(A6,"mm")</f>
-        <v>08</v>
+        <v>09</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
         <f ca="1">TEXT(A6,"m")</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="str">
         <f ca="1">TEXT(A12,"mmm-yy")</f>
-        <v>Aug-26</v>
+        <v>Sep-26</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20">
         <f ca="1">WEEKDAY(A12,11)</f>
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="41">
+      <c r="A21" s="40">
         <v>46113</v>
       </c>
-      <c r="B21" s="41">
+      <c r="B21" s="40">
         <v>46326</v>
       </c>
       <c r="C21">
@@ -3710,19 +4825,19 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B24" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="B25" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="41">
+      <c r="A27" s="40">
         <v>46113</v>
       </c>
-      <c r="B27" s="41">
+      <c r="B27" s="40">
         <v>46249</v>
       </c>
       <c r="C27">
@@ -3743,31 +4858,31 @@
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="41">
+      <c r="A31" s="40">
         <v>46127</v>
       </c>
       <c r="B31">
         <v>6</v>
       </c>
-      <c r="C31" s="41">
+      <c r="C31" s="40">
         <f>EDATE(A31,B31)</f>
         <v>46310</v>
       </c>
       <c r="D31" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="C32" s="41">
+      <c r="C32" s="40">
         <f>EOMONTH(A31,B31)</f>
         <v>46326</v>
       </c>
       <c r="D32" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" s="41">
+      <c r="A33" s="40">
         <v>46127</v>
       </c>
       <c r="B33">
@@ -3776,19 +4891,19 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" s="41">
+      <c r="A38" s="40">
         <v>46113</v>
       </c>
-      <c r="B38" s="41">
+      <c r="B38" s="40">
         <v>46326</v>
       </c>
       <c r="C38">
@@ -3796,25 +4911,29 @@
         <v>213</v>
       </c>
       <c r="D38" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E38" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="F38" t="s">
-        <v>234</v>
-      </c>
+        <v>232</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B39" s="51"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="B40" s="40"/>
       <c r="C40">
         <f>NETWORKDAYS.INTL(A38,B38,11,)</f>
         <v>184</v>
       </c>
       <c r="D40" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="E40" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
     </row>
   </sheetData>
@@ -3865,12 +4984,15 @@
       <c r="D2" s="1">
         <v>15000</v>
       </c>
-      <c r="E2" s="1"/>
+      <c r="E2" s="1">
+        <f>IF(C2=$I$4,$J$4,IF(C2=$I$6,$J$6,IF(C2=$I$8,$J$8,IF(C2=$I$10,$J$10,0))))</f>
+        <v>5000</v>
+      </c>
       <c r="P2" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="Q2" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
@@ -3886,12 +5008,15 @@
       <c r="D3" s="1">
         <v>16000</v>
       </c>
-      <c r="E3" s="1"/>
+      <c r="E3" s="1">
+        <f t="shared" ref="E3:E13" si="0">IF(C3=$I$4,$J$4,IF(C3=$I$6,$J$6,IF(C3=$I$8,$J$8,IF(C3=$I$10,$J$10,0))))</f>
+        <v>3000</v>
+      </c>
       <c r="P3" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="Q3" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
@@ -3907,7 +5032,10 @@
       <c r="D4" s="1">
         <v>18000</v>
       </c>
-      <c r="E4" s="1"/>
+      <c r="E4" s="1">
+        <f t="shared" si="0"/>
+        <v>5000</v>
+      </c>
       <c r="I4" s="1" t="s">
         <v>61</v>
       </c>
@@ -3915,10 +5043,10 @@
         <v>5000</v>
       </c>
       <c r="P4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="Q4" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -3934,11 +5062,14 @@
       <c r="D5" s="1">
         <v>19000</v>
       </c>
-      <c r="E5" s="1"/>
+      <c r="E5" s="1">
+        <f t="shared" si="0"/>
+        <v>2000</v>
+      </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1"/>
       <c r="Q5" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
@@ -3954,7 +5085,10 @@
       <c r="D6" s="1">
         <v>25000</v>
       </c>
-      <c r="E6" s="1"/>
+      <c r="E6" s="1">
+        <f t="shared" si="0"/>
+        <v>2500</v>
+      </c>
       <c r="I6" s="1" t="s">
         <v>62</v>
       </c>
@@ -3975,7 +5109,10 @@
       <c r="D7" s="1">
         <v>22000</v>
       </c>
-      <c r="E7" s="1"/>
+      <c r="E7" s="1">
+        <f t="shared" si="0"/>
+        <v>5000</v>
+      </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1"/>
     </row>
@@ -3992,7 +5129,10 @@
       <c r="D8" s="1">
         <v>15000</v>
       </c>
-      <c r="E8" s="1"/>
+      <c r="E8" s="1">
+        <f t="shared" si="0"/>
+        <v>3000</v>
+      </c>
       <c r="I8" s="1" t="s">
         <v>64</v>
       </c>
@@ -4008,12 +5148,15 @@
         <v>8</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="D9" s="1">
         <v>35000</v>
       </c>
-      <c r="E9" s="1"/>
+      <c r="E9" s="1">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1"/>
     </row>
@@ -4030,7 +5173,10 @@
       <c r="D10" s="1">
         <v>15000</v>
       </c>
-      <c r="E10" s="1"/>
+      <c r="E10" s="1">
+        <f t="shared" si="0"/>
+        <v>2500</v>
+      </c>
       <c r="I10" s="1" t="s">
         <v>63</v>
       </c>
@@ -4051,7 +5197,10 @@
       <c r="D11" s="1">
         <v>35000</v>
       </c>
-      <c r="E11" s="1"/>
+      <c r="E11" s="1">
+        <f t="shared" si="0"/>
+        <v>2500</v>
+      </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
@@ -4066,7 +5215,10 @@
       <c r="D12" s="1">
         <v>18000</v>
       </c>
-      <c r="E12" s="1"/>
+      <c r="E12" s="1">
+        <f t="shared" si="0"/>
+        <v>2500</v>
+      </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
@@ -4081,7 +5233,10 @@
       <c r="D13" s="1">
         <v>21000</v>
       </c>
-      <c r="E13" s="1"/>
+      <c r="E13" s="1">
+        <f t="shared" si="0"/>
+        <v>2500</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4117,16 +5272,18 @@
       <c r="E1" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="F1" s="22"/>
-      <c r="G1" s="24"/>
-      <c r="H1" s="24" t="s">
+      <c r="F1" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23" t="s">
         <v>60</v>
       </c>
-      <c r="I1" s="24" t="s">
+      <c r="I1" s="23" t="s">
         <v>113</v>
       </c>
-      <c r="J1" s="24" t="s">
-        <v>238</v>
+      <c r="J1" s="23" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.25">
@@ -4142,15 +5299,22 @@
       <c r="D2" s="1">
         <v>15000</v>
       </c>
-      <c r="E2" s="1"/>
+      <c r="E2" s="1" t="str">
+        <f>IF(AND(C2=$H$2,D2&gt;=$I$2),$J$2,$J$3)</f>
+        <v>no</v>
+      </c>
+      <c r="F2" s="1" t="str">
+        <f>IF(OR(C2=$H$2,D2&gt;=$I$2),$J$2,$J$3)</f>
+        <v>yes</v>
+      </c>
       <c r="H2" t="s">
         <v>61</v>
       </c>
-      <c r="I2" t="s">
-        <v>114</v>
+      <c r="I2">
+        <v>20000</v>
       </c>
       <c r="J2" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -4166,9 +5330,16 @@
       <c r="D3" s="1">
         <v>16000</v>
       </c>
-      <c r="E3" s="1"/>
+      <c r="E3" s="1" t="str">
+        <f t="shared" ref="E3:E13" si="0">IF(AND(C3=$H$2,D3&gt;=$I$2),$J$2,$J$3)</f>
+        <v>no</v>
+      </c>
+      <c r="F3" s="1" t="str">
+        <f t="shared" ref="F3:F13" si="1">IF(OR(C3=$H$2,D3&gt;=$I$2),$J$2,$J$3)</f>
+        <v>no</v>
+      </c>
       <c r="J3" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -4184,7 +5355,14 @@
       <c r="D4" s="1">
         <v>18000</v>
       </c>
-      <c r="E4" s="1"/>
+      <c r="E4" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>no</v>
+      </c>
+      <c r="F4" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>yes</v>
+      </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -4199,9 +5377,16 @@
       <c r="D5" s="1">
         <v>19000</v>
       </c>
-      <c r="E5" s="1"/>
+      <c r="E5" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>no</v>
+      </c>
+      <c r="F5" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>no</v>
+      </c>
       <c r="H5" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -4217,9 +5402,16 @@
       <c r="D6" s="1">
         <v>25000</v>
       </c>
-      <c r="E6" s="1"/>
+      <c r="E6" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>no</v>
+      </c>
+      <c r="F6" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>yes</v>
+      </c>
       <c r="H6" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -4235,9 +5427,16 @@
       <c r="D7" s="1">
         <v>22000</v>
       </c>
-      <c r="E7" s="1"/>
+      <c r="E7" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>yes</v>
+      </c>
+      <c r="F7" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>yes</v>
+      </c>
       <c r="H7" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -4253,7 +5452,14 @@
       <c r="D8" s="1">
         <v>15000</v>
       </c>
-      <c r="E8" s="1"/>
+      <c r="E8" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>no</v>
+      </c>
+      <c r="F8" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>no</v>
+      </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -4268,7 +5474,14 @@
       <c r="D9" s="1">
         <v>35000</v>
       </c>
-      <c r="E9" s="1"/>
+      <c r="E9" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>yes</v>
+      </c>
+      <c r="F9" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>yes</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -4283,7 +5496,14 @@
       <c r="D10" s="1">
         <v>15000</v>
       </c>
-      <c r="E10" s="1"/>
+      <c r="E10" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>no</v>
+      </c>
+      <c r="F10" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>no</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
@@ -4298,7 +5518,14 @@
       <c r="D11" s="1">
         <v>35000</v>
       </c>
-      <c r="E11" s="1"/>
+      <c r="E11" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>no</v>
+      </c>
+      <c r="F11" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>yes</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
@@ -4313,7 +5540,14 @@
       <c r="D12" s="1">
         <v>18000</v>
       </c>
-      <c r="E12" s="1"/>
+      <c r="E12" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>no</v>
+      </c>
+      <c r="F12" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>no</v>
+      </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
@@ -4328,7 +5562,14 @@
       <c r="D13" s="1">
         <v>21000</v>
       </c>
-      <c r="E13" s="1"/>
+      <c r="E13" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>no</v>
+      </c>
+      <c r="F13" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>yes</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4338,7 +5579,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:W15"/>
+  <dimension ref="A1:X15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -4347,35 +5588,35 @@
     <col min="23" max="23" width="9.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="1:23" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:24" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <f>COUNT(C3:T15)</f>
         <v>0</v>
       </c>
-      <c r="C2" s="52" t="s">
+      <c r="C2" s="58" t="s">
         <v>40</v>
       </c>
-      <c r="D2" s="53"/>
-      <c r="E2" s="53"/>
-      <c r="F2" s="53"/>
-      <c r="G2" s="53"/>
-      <c r="H2" s="53"/>
-      <c r="I2" s="53"/>
-      <c r="J2" s="53"/>
-      <c r="K2" s="53"/>
-      <c r="L2" s="53"/>
-      <c r="M2" s="53"/>
-      <c r="N2" s="53"/>
-      <c r="O2" s="53"/>
-      <c r="P2" s="53"/>
-      <c r="Q2" s="53"/>
-      <c r="R2" s="53"/>
-      <c r="S2" s="53"/>
-      <c r="T2" s="53"/>
-      <c r="U2" s="54"/>
-    </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="D2" s="59"/>
+      <c r="E2" s="59"/>
+      <c r="F2" s="59"/>
+      <c r="G2" s="59"/>
+      <c r="H2" s="59"/>
+      <c r="I2" s="59"/>
+      <c r="J2" s="59"/>
+      <c r="K2" s="59"/>
+      <c r="L2" s="59"/>
+      <c r="M2" s="59"/>
+      <c r="N2" s="59"/>
+      <c r="O2" s="59"/>
+      <c r="P2" s="59"/>
+      <c r="Q2" s="59"/>
+      <c r="R2" s="59"/>
+      <c r="S2" s="59"/>
+      <c r="T2" s="59"/>
+      <c r="U2" s="60"/>
+    </row>
+    <row r="3" spans="1:24" x14ac:dyDescent="0.25">
       <c r="A3">
         <f>COUNTA(C3:U15,)</f>
         <v>137</v>
@@ -4440,8 +5681,12 @@
       <c r="W3" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="X3">
+        <f>COUNTA(C3:U15)</f>
+        <v>136</v>
+      </c>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C4" s="1" t="s">
         <v>46</v>
       </c>
@@ -4484,8 +5729,12 @@
       <c r="W4" t="s">
         <v>42</v>
       </c>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="X4">
+        <f>COUNTBLANK(C3:U15)</f>
+        <v>111</v>
+      </c>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C5" s="1" t="s">
         <v>45</v>
       </c>
@@ -4528,7 +5777,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C6" s="1" t="s">
         <v>46</v>
       </c>
@@ -4570,11 +5819,18 @@
       <c r="U6" s="1" t="s">
         <v>46</v>
       </c>
+      <c r="V6" s="21" t="s">
+        <v>46</v>
+      </c>
       <c r="W6" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="X6">
+        <f>COUNTIF(C3:U15,V6)</f>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C7" s="1" t="s">
         <v>45</v>
       </c>
@@ -4610,11 +5866,18 @@
       <c r="U7" s="1" t="s">
         <v>45</v>
       </c>
+      <c r="V7" s="21" t="s">
+        <v>45</v>
+      </c>
       <c r="W7" t="s">
         <v>44</v>
       </c>
-    </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="X7">
+        <f>COUNTIF(C3:U15,V7)</f>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="8" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C8" s="1" t="s">
         <v>45</v>
       </c>
@@ -4661,7 +5924,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C9" s="1" t="s">
         <v>45</v>
       </c>
@@ -4708,7 +5971,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C10" s="1" t="s">
         <v>45</v>
       </c>
@@ -4763,7 +6026,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C11" s="1" t="s">
         <v>46</v>
       </c>
@@ -4804,7 +6067,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C12" s="1" t="s">
         <v>46</v>
       </c>
@@ -4837,7 +6100,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C13" s="1" t="s">
         <v>46</v>
       </c>
@@ -4870,7 +6133,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C14" s="1" t="s">
         <v>46</v>
       </c>
@@ -4903,7 +6166,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.25">
       <c r="C15" s="1" t="s">
         <v>46</v>
       </c>
@@ -4940,11 +6203,11 @@
   <mergeCells count="1">
     <mergeCell ref="C2:U2"/>
   </mergeCells>
-  <conditionalFormatting sqref="C3:U15">
-    <cfRule type="cellIs" dxfId="7" priority="1" operator="equal">
+  <conditionalFormatting sqref="C3:U15 V6:V7">
+    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
       <formula>"M"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
       <formula>"F"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4965,17 +6228,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="45" t="s">
+      <c r="A1" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="45" t="s">
         <v>14</v>
       </c>
-      <c r="C1" s="47" t="s">
+      <c r="C1" s="46" t="s">
         <v>15</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>17</v>
+      </c>
+      <c r="F1">
+        <f>SUMIF($B$2:$B$16,E1,$C$2:$C$16)</f>
+        <v>245658</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
@@ -4985,11 +6252,15 @@
       <c r="B2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C2" s="28">
+      <c r="C2" s="27">
         <v>34133</v>
       </c>
       <c r="E2" s="1" t="s">
         <v>19</v>
+      </c>
+      <c r="F2">
+        <f>SUMIF($B$2:$B$16,E2,$C$2:$C$16)</f>
+        <v>88647</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -4999,11 +6270,15 @@
       <c r="B3" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C3" s="28">
+      <c r="C3" s="27">
         <v>30861</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>21</v>
+      </c>
+      <c r="F3">
+        <f>SUMIF($B$2:$B$16,E3,$C$2:$C$16)</f>
+        <v>160145</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
@@ -5013,7 +6288,7 @@
       <c r="B4" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C4" s="28">
+      <c r="C4" s="27">
         <v>26895</v>
       </c>
     </row>
@@ -5024,7 +6299,7 @@
       <c r="B5" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C5" s="28">
+      <c r="C5" s="27">
         <v>29264</v>
       </c>
     </row>
@@ -5035,7 +6310,7 @@
       <c r="B6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="28">
+      <c r="C6" s="27">
         <v>36505</v>
       </c>
     </row>
@@ -5046,10 +6321,10 @@
       <c r="B7" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="27">
         <v>30041</v>
       </c>
-      <c r="G7" s="27"/>
+      <c r="G7" s="26"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="15" t="s">
@@ -5058,7 +6333,7 @@
       <c r="B8" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C8" s="28">
+      <c r="C8" s="27">
         <v>34141</v>
       </c>
     </row>
@@ -5069,7 +6344,7 @@
       <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="28">
+      <c r="C9" s="27">
         <v>32914</v>
       </c>
     </row>
@@ -5080,7 +6355,7 @@
       <c r="B10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="28">
+      <c r="C10" s="27">
         <v>37908</v>
       </c>
     </row>
@@ -5091,7 +6366,7 @@
       <c r="B11" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C11" s="28">
+      <c r="C11" s="27">
         <v>28875</v>
       </c>
     </row>
@@ -5102,7 +6377,7 @@
       <c r="B12" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C12" s="28">
+      <c r="C12" s="27">
         <v>36135</v>
       </c>
     </row>
@@ -5113,108 +6388,108 @@
       <c r="B13" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="27">
         <v>31711</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="44" t="s">
-        <v>200</v>
+      <c r="A14" s="43" t="s">
+        <v>198</v>
       </c>
       <c r="B14" s="21" t="s">
         <v>17</v>
       </c>
-      <c r="C14" s="28">
+      <c r="C14" s="27">
         <v>38791</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="44" t="s">
-        <v>201</v>
+      <c r="A15" s="43" t="s">
+        <v>199</v>
       </c>
       <c r="B15" s="21" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="28">
+      <c r="C15" s="27">
         <v>38598</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="48" t="s">
-        <v>202</v>
-      </c>
-      <c r="B16" s="49" t="s">
+      <c r="A16" s="47" t="s">
+        <v>200</v>
+      </c>
+      <c r="B16" s="48" t="s">
         <v>21</v>
       </c>
-      <c r="C16" s="28">
+      <c r="C16" s="27">
         <v>27678</v>
       </c>
     </row>
     <row r="18" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C18" s="29"/>
-      <c r="D18" s="32"/>
-      <c r="G18" s="31"/>
+      <c r="C18" s="28"/>
+      <c r="D18" s="31"/>
+      <c r="G18" s="30"/>
     </row>
     <row r="19" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C19" s="29"/>
-      <c r="D19" s="32"/>
-      <c r="G19" s="31"/>
+      <c r="C19" s="28"/>
+      <c r="D19" s="31"/>
+      <c r="G19" s="30"/>
     </row>
     <row r="20" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C20" s="29"/>
-      <c r="D20" s="32"/>
-      <c r="E20" s="30"/>
-      <c r="G20" s="31"/>
+      <c r="C20" s="28"/>
+      <c r="D20" s="31"/>
+      <c r="E20" s="29"/>
+      <c r="G20" s="30"/>
     </row>
     <row r="21" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C21" s="29"/>
-      <c r="D21" s="32"/>
-      <c r="E21" s="30"/>
-      <c r="G21" s="31"/>
+      <c r="C21" s="28"/>
+      <c r="D21" s="31"/>
+      <c r="E21" s="29"/>
+      <c r="G21" s="30"/>
     </row>
     <row r="22" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C22" s="29"/>
-      <c r="D22" s="32"/>
-      <c r="E22" s="30"/>
-      <c r="G22" s="31"/>
+      <c r="C22" s="28"/>
+      <c r="D22" s="31"/>
+      <c r="E22" s="29"/>
+      <c r="G22" s="30"/>
     </row>
     <row r="23" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C23" s="29"/>
-      <c r="D23" s="32"/>
-      <c r="E23" s="30"/>
-      <c r="G23" s="31"/>
+      <c r="C23" s="28"/>
+      <c r="D23" s="31"/>
+      <c r="E23" s="29"/>
+      <c r="G23" s="30"/>
     </row>
     <row r="24" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C24" s="29"/>
-      <c r="D24" s="33"/>
-      <c r="E24" s="30"/>
-      <c r="G24" s="31"/>
+      <c r="C24" s="28"/>
+      <c r="D24" s="32"/>
+      <c r="E24" s="29"/>
+      <c r="G24" s="30"/>
     </row>
     <row r="25" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C25" s="29"/>
-      <c r="D25" s="33"/>
-      <c r="E25" s="30"/>
-      <c r="G25" s="31"/>
+      <c r="C25" s="28"/>
+      <c r="D25" s="32"/>
+      <c r="E25" s="29"/>
+      <c r="G25" s="30"/>
     </row>
     <row r="26" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="C26" s="29"/>
-      <c r="D26" s="33"/>
-      <c r="E26" s="30"/>
-      <c r="G26" s="31"/>
+      <c r="C26" s="28"/>
+      <c r="D26" s="32"/>
+      <c r="E26" s="29"/>
+      <c r="G26" s="30"/>
     </row>
     <row r="27" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D27" s="33"/>
-      <c r="E27" s="30"/>
-      <c r="G27" s="31"/>
+      <c r="D27" s="32"/>
+      <c r="E27" s="29"/>
+      <c r="G27" s="30"/>
     </row>
     <row r="28" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D28" s="33"/>
+      <c r="D28" s="32"/>
     </row>
     <row r="29" spans="3:7" x14ac:dyDescent="0.25">
-      <c r="D29" s="33"/>
+      <c r="D29" s="32"/>
     </row>
   </sheetData>
-  <sortState ref="A2:C13">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C13">
     <sortCondition ref="B2"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -5275,8 +6550,14 @@
       <c r="F2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="G2" s="1">
+        <f>SUMIFS($D$2:$D$13,$B$2:$B$13,F2,$C$2:$C$13,$G$1)</f>
+        <v>4500</v>
+      </c>
+      <c r="H2" s="1">
+        <f>SUMIFS($D$2:$D$13,$B$2:$B$13,F2,$C$2:$C$13,$H$1)</f>
+        <v>5150</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -5294,8 +6575,14 @@
       <c r="F3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="G3" s="1">
+        <f>SUMIFS($D$2:$D$13,$B$2:$B$13,F3,$C$2:$C$13,$G$1)</f>
+        <v>11500</v>
+      </c>
+      <c r="H3" s="1">
+        <f t="shared" ref="H3:H4" si="0">SUMIFS($D$2:$D$13,$B$2:$B$13,F3,$C$2:$C$13,$H$1)</f>
+        <v>11100</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -5313,8 +6600,14 @@
       <c r="F4" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="G4" s="1">
+        <f t="shared" ref="G4" si="1">SUMIFS($D$2:$D$13,$B$2:$B$13,F4,$C$2:$C$13,$G$1)</f>
+        <v>8950</v>
+      </c>
+      <c r="H4" s="1">
+        <f t="shared" si="0"/>
+        <v>2560</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -5380,7 +6673,10 @@
       <c r="F8" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G8" s="1"/>
+      <c r="G8" s="1">
+        <f>SUMIF($B$2:$B$13,F8,$D$2:$D$13)</f>
+        <v>9650</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
@@ -5398,7 +6694,10 @@
       <c r="F9" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G9" s="1"/>
+      <c r="G9" s="1">
+        <f t="shared" ref="G9:G10" si="2">SUMIF($B$2:$B$13,F9,$D$2:$D$13)</f>
+        <v>22600</v>
+      </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -5416,7 +6715,10 @@
       <c r="F10" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="G10" s="1"/>
+      <c r="G10" s="1">
+        <f t="shared" si="2"/>
+        <v>11510</v>
+      </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
@@ -5437,7 +6739,7 @@
         <v>43739</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>37</v>
@@ -5470,26 +6772,34 @@
       <c r="F14" s="1" t="s">
         <v>37</v>
       </c>
+      <c r="G14" s="1">
+        <f>SUMIF($C$2:$C$13,F14,$D$2:$D$13)</f>
+        <v>24950</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="F15" s="1" t="s">
         <v>38</v>
       </c>
+      <c r="G15" s="1">
+        <f>SUMIF($C$2:$C$13,F15,$D$2:$D$13)</f>
+        <v>18810</v>
+      </c>
     </row>
     <row r="17" spans="6:7" x14ac:dyDescent="0.25">
-      <c r="G17" s="25"/>
+      <c r="G17" s="24"/>
     </row>
     <row r="18" spans="6:7" x14ac:dyDescent="0.25">
-      <c r="F18" s="25"/>
+      <c r="F18" s="24"/>
     </row>
     <row r="39" spans="3:6" x14ac:dyDescent="0.25">
-      <c r="C39" s="26"/>
-      <c r="D39" s="26"/>
-      <c r="E39" s="26"/>
-      <c r="F39" s="26"/>
+      <c r="C39" s="25"/>
+      <c r="D39" s="25"/>
+      <c r="E39" s="25"/>
+      <c r="F39" s="25"/>
     </row>
   </sheetData>
-  <sortState ref="A2:D13">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D13">
     <sortCondition ref="B2:B13"/>
     <sortCondition ref="C2:C13"/>
     <sortCondition descending="1" ref="D2:D13"/>
@@ -5545,13 +6855,16 @@
       <c r="C2" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D2" s="40">
+      <c r="D2" s="39">
         <v>600</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="1"/>
+      <c r="G2" s="1">
+        <f>COUNTIF($B$2:$B$13,F2)</f>
+        <v>4</v>
+      </c>
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
@@ -5564,13 +6877,16 @@
       <c r="C3" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D3" s="40">
+      <c r="D3" s="39">
         <v>4500</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="1"/>
+      <c r="G3" s="1">
+        <f t="shared" ref="G3:G4" si="0">COUNTIF($B$2:$B$13,F3)</f>
+        <v>4</v>
+      </c>
       <c r="H3" s="1"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -5583,13 +6899,16 @@
       <c r="C4" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D4" s="40">
+      <c r="D4" s="39">
         <v>6000</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="G4" s="1"/>
+      <c r="G4" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
@@ -5602,7 +6921,7 @@
       <c r="C5" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D5" s="40">
+      <c r="D5" s="39">
         <v>6500</v>
       </c>
     </row>
@@ -5616,7 +6935,7 @@
       <c r="C6" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="40">
+      <c r="D6" s="39">
         <v>1450</v>
       </c>
     </row>
@@ -5630,14 +6949,14 @@
       <c r="C7" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D7" s="40">
+      <c r="D7" s="39">
         <v>1500</v>
       </c>
       <c r="F7" s="3" t="s">
         <v>33</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
@@ -5650,11 +6969,15 @@
       <c r="C8" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D8" s="40">
+      <c r="D8" s="39">
         <v>2560</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>37</v>
+      </c>
+      <c r="G8" s="1">
+        <f>COUNTIF($C$2:$C$13,F8)</f>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
@@ -5667,11 +6990,15 @@
       <c r="C9" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="40">
+      <c r="D9" s="39">
         <v>6000</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>38</v>
+      </c>
+      <c r="G9" s="1">
+        <f>COUNTIF($C$2:$C$13,F9)</f>
+        <v>5</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
@@ -5684,7 +7011,7 @@
       <c r="C10" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D10" s="40">
+      <c r="D10" s="39">
         <v>650</v>
       </c>
     </row>
@@ -5698,7 +7025,7 @@
       <c r="C11" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D11" s="40">
+      <c r="D11" s="39">
         <v>4500</v>
       </c>
     </row>
@@ -5712,7 +7039,7 @@
       <c r="C12" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="40">
+      <c r="D12" s="39">
         <v>4500</v>
       </c>
     </row>
@@ -5726,249 +7053,249 @@
       <c r="C13" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D13" s="40">
+      <c r="D13" s="39">
         <v>5000</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="33"/>
-      <c r="F19" s="37">
+      <c r="A19" s="32"/>
+      <c r="F19" s="36">
         <v>11</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="33"/>
+      <c r="A20" s="32"/>
       <c r="F20">
         <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="33"/>
+      <c r="A21" s="32"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="33"/>
+      <c r="A22" s="32"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="33"/>
+      <c r="A23" s="32"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="33" t="s">
-        <v>140</v>
-      </c>
-      <c r="F24" s="38">
-        <f t="shared" ref="D24:G35" ca="1" si="0">RANDBETWEEN(5000,50000)</f>
-        <v>13072</v>
-      </c>
-      <c r="G24" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>20139</v>
+      <c r="A24" s="32" t="s">
+        <v>139</v>
+      </c>
+      <c r="F24" s="37">
+        <f t="shared" ref="D24:G35" ca="1" si="1">RANDBETWEEN(5000,50000)</f>
+        <v>17753</v>
+      </c>
+      <c r="G24" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>27938</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>139</v>
-      </c>
-      <c r="C25" s="36">
+        <v>138</v>
+      </c>
+      <c r="C25" s="35">
         <v>43922</v>
       </c>
       <c r="D25" t="s">
+        <v>141</v>
+      </c>
+      <c r="E25" t="s">
         <v>142</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>38991</v>
+      </c>
+      <c r="G25" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>5183</v>
+      </c>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A26" s="32" t="s">
+        <v>137</v>
+      </c>
+      <c r="C26" s="34"/>
+      <c r="E26" t="s">
         <v>143</v>
       </c>
-      <c r="F25" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>42833</v>
-      </c>
-      <c r="G25" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>26623</v>
-      </c>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="33" t="s">
-        <v>138</v>
-      </c>
-      <c r="C26" s="35"/>
-      <c r="E26" t="s">
-        <v>144</v>
-      </c>
-      <c r="F26" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>47537</v>
-      </c>
-      <c r="G26" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>11022</v>
+      <c r="F26" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>38765</v>
+      </c>
+      <c r="G26" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>18673</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>141</v>
-      </c>
-      <c r="C27" s="35"/>
+        <v>140</v>
+      </c>
+      <c r="C27" s="34"/>
       <c r="E27" t="s">
+        <v>144</v>
+      </c>
+      <c r="F27" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>16273</v>
+      </c>
+      <c r="G27" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>28442</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A28" s="32"/>
+      <c r="C28" s="34"/>
+      <c r="E28" t="s">
         <v>145</v>
       </c>
-      <c r="F27" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>35730</v>
-      </c>
-      <c r="G27" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>33489</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="33"/>
-      <c r="C28" s="35"/>
-      <c r="E28" t="s">
+      <c r="F28" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>14912</v>
+      </c>
+      <c r="G28" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>16252</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A29" s="32"/>
+      <c r="C29" s="34"/>
+      <c r="F29" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>16425</v>
+      </c>
+      <c r="G29" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>11897</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A30" s="32"/>
+      <c r="C30" s="37">
+        <f ca="1">RANDBETWEEN(5000,50000)</f>
+        <v>47671</v>
+      </c>
+      <c r="D30" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>11434</v>
+      </c>
+      <c r="E30" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>12314</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A31" s="32"/>
+      <c r="C31" s="37">
+        <f t="shared" ref="C31:C35" ca="1" si="2">RANDBETWEEN(5000,50000)</f>
+        <v>39568</v>
+      </c>
+      <c r="D31" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>42827</v>
+      </c>
+      <c r="E31" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>43341</v>
+      </c>
+      <c r="G31" s="38" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A32" s="32"/>
+      <c r="C32" s="37">
+        <f t="shared" ca="1" si="2"/>
+        <v>45471</v>
+      </c>
+      <c r="D32" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>38349</v>
+      </c>
+      <c r="E32" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>7219</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" s="32"/>
+      <c r="C33" s="37">
+        <f t="shared" ca="1" si="2"/>
+        <v>12859</v>
+      </c>
+      <c r="D33" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>33386</v>
+      </c>
+      <c r="E33" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>14240</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" s="33"/>
+      <c r="C34" s="37">
+        <f t="shared" ca="1" si="2"/>
+        <v>41396</v>
+      </c>
+      <c r="D34" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>33252</v>
+      </c>
+      <c r="E34" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>26332</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" s="33"/>
+      <c r="C35" s="37">
+        <f t="shared" ca="1" si="2"/>
+        <v>11149</v>
+      </c>
+      <c r="D35" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>26414</v>
+      </c>
+      <c r="E35" s="37">
+        <f t="shared" ca="1" si="1"/>
+        <v>40592</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" s="33"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="33"/>
+      <c r="D37" t="s">
         <v>146</v>
       </c>
-      <c r="F28" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>36939</v>
-      </c>
-      <c r="G28" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>27128</v>
-      </c>
-    </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="33"/>
-      <c r="C29" s="35"/>
-      <c r="F29" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>37837</v>
-      </c>
-      <c r="G29" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>45525</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="33"/>
-      <c r="C30" s="38">
-        <f ca="1">RANDBETWEEN(5000,50000)</f>
-        <v>44443</v>
-      </c>
-      <c r="D30" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>35197</v>
-      </c>
-      <c r="E30" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>7927</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="21" x14ac:dyDescent="0.35">
-      <c r="A31" s="33"/>
-      <c r="C31" s="38">
-        <f t="shared" ref="C31:C35" ca="1" si="1">RANDBETWEEN(5000,50000)</f>
-        <v>40796</v>
-      </c>
-      <c r="D31" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>28881</v>
-      </c>
-      <c r="E31" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>16302</v>
-      </c>
-      <c r="G31" s="39" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="33"/>
-      <c r="C32" s="38">
-        <f t="shared" ca="1" si="1"/>
-        <v>8089</v>
-      </c>
-      <c r="D32" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>6895</v>
-      </c>
-      <c r="E32" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>6028</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="33"/>
-      <c r="C33" s="38">
-        <f t="shared" ca="1" si="1"/>
-        <v>14143</v>
-      </c>
-      <c r="D33" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>26770</v>
-      </c>
-      <c r="E33" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>38279</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="34"/>
-      <c r="C34" s="38">
-        <f t="shared" ca="1" si="1"/>
-        <v>43445</v>
-      </c>
-      <c r="D34" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>11845</v>
-      </c>
-      <c r="E34" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>12726</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="34"/>
-      <c r="C35" s="38">
-        <f t="shared" ca="1" si="1"/>
-        <v>41977</v>
-      </c>
-      <c r="D35" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>33719</v>
-      </c>
-      <c r="E35" s="38">
-        <f t="shared" ca="1" si="0"/>
-        <v>8915</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="34"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="34"/>
-      <c r="D37" t="s">
+      <c r="E37" t="s">
         <v>147</v>
       </c>
-      <c r="E37" t="s">
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A38" s="33"/>
+      <c r="D38" t="s">
         <v>148</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="34"/>
-      <c r="D38" t="s">
+      <c r="E38" t="s">
         <v>149</v>
       </c>
-      <c r="E38" t="s">
-        <v>150</v>
-      </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="34"/>
+      <c r="A39" s="33"/>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="34"/>
+      <c r="A40" s="33"/>
     </row>
   </sheetData>
-  <sortState ref="A2:D11">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D11">
     <sortCondition ref="B2"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -6026,8 +7353,14 @@
       <c r="F2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="G2" s="1">
+        <f>COUNTIFS($B$2:$B$13,F2,$C$2:$C$13,$G$1)</f>
+        <v>2</v>
+      </c>
+      <c r="H2" s="1">
+        <f>COUNTIFS($B$2:$B$13,F2,$C$2:$C$13,$H$1)</f>
+        <v>2</v>
+      </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
@@ -6045,8 +7378,14 @@
       <c r="F3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="G3" s="1">
+        <f t="shared" ref="G3:G4" si="0">COUNTIFS($B$2:$B$13,F3,$C$2:$C$13,$G$1)</f>
+        <v>1</v>
+      </c>
+      <c r="H3" s="1">
+        <f t="shared" ref="H3:H4" si="1">COUNTIFS($B$2:$B$13,F3,$C$2:$C$13,$H$1)</f>
+        <v>3</v>
+      </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
@@ -6064,8 +7403,14 @@
       <c r="F4" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="G4" s="1">
+        <f t="shared" si="0"/>
+        <v>4</v>
+      </c>
+      <c r="H4" s="1">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
@@ -6249,8 +7594,14 @@
       <c r="F2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="G2" s="1">
+        <f>AVERAGEIFS($D$2:$D$13,$B$2:$B$13,F2,$C$2:$C$13,$G$1)</f>
+        <v>4750</v>
+      </c>
+      <c r="H2" s="1">
+        <f>AVERAGEIFS($D$2:$D$13,$B$2:$B$13,F2,$C$2:$C$13,$H$1)</f>
+        <v>2575</v>
+      </c>
       <c r="J2" s="1"/>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -6269,8 +7620,14 @@
       <c r="F3" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="G3" s="1">
+        <f t="shared" ref="G3:G4" si="0">AVERAGEIFS($D$2:$D$13,$B$2:$B$13,F3,$C$2:$C$13,$G$1)</f>
+        <v>6500</v>
+      </c>
+      <c r="H3" s="1">
+        <f t="shared" ref="H3" si="1">AVERAGEIFS($D$2:$D$13,$B$2:$B$13,F3,$C$2:$C$13,$H$1)</f>
+        <v>3700</v>
+      </c>
       <c r="J3" s="1"/>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -6287,10 +7644,16 @@
         <v>4500</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+        <v>36</v>
+      </c>
+      <c r="G4" s="1">
+        <f t="shared" si="0"/>
+        <v>2877.5</v>
+      </c>
+      <c r="H4" s="1" t="e">
+        <f>AVERAGEIFS($D$2:$D$13,$B$2:$B$13,F4,$C$2:$C$13,$H$1)</f>
+        <v>#DIV/0!</v>
+      </c>
       <c r="J4" s="1"/>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -6371,7 +7734,10 @@
       <c r="F9" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="G9" s="1"/>
+      <c r="G9" s="1">
+        <f>AVERAGEIF($B$2:$B$13,F9,$D$2:$D$13)</f>
+        <v>3662.5</v>
+      </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
@@ -6389,7 +7755,10 @@
       <c r="F10" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="G10" s="1"/>
+      <c r="G10" s="1">
+        <f t="shared" ref="G10:G11" si="2">AVERAGEIF($B$2:$B$13,F10,$D$2:$D$13)</f>
+        <v>4400</v>
+      </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
@@ -6407,7 +7776,10 @@
       <c r="F11" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="G11" s="1"/>
+      <c r="G11" s="1">
+        <f t="shared" si="2"/>
+        <v>2877.5</v>
+      </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
@@ -6449,10 +7821,18 @@
       <c r="F15" s="1" t="s">
         <v>37</v>
       </c>
+      <c r="G15" s="1">
+        <f>AVERAGEIF($C$2:$C$13,F15,$D$2:$D$13)</f>
+        <v>3930</v>
+      </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
       <c r="F16" s="1" t="s">
         <v>38</v>
+      </c>
+      <c r="G16" s="1">
+        <f>AVERAGEIF($C$2:$C$13,F16,$D$2:$D$13)</f>
+        <v>3250</v>
       </c>
     </row>
   </sheetData>

</xml_diff>